<commit_message>
Cap nhat he thong tu dong hoa Dusk
</commit_message>
<xml_diff>
--- a/tests/Browser/Excel/DiemDanh.xlsx
+++ b/tests/Browser/Excel/DiemDanh.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\TuDongLamViec\tests\Browser\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8EEE03-2B9C-45A4-B991-DB8291235D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC506237-1570-4AFF-BF54-DBFFDA174B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8330" yWindow="1840" windowWidth="19200" windowHeight="10060" xr2:uid="{06A80A3C-E8BE-424B-9614-FA41F15A8077}"/>
+    <workbookView xWindow="3980" yWindow="2830" windowWidth="19200" windowHeight="10060" xr2:uid="{06A80A3C-E8BE-424B-9614-FA41F15A8077}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="76">
   <si>
     <t>ten_cuoc_hop</t>
   </si>
@@ -33,31 +33,226 @@
     <t>ten_dai_bieu</t>
   </si>
   <si>
-    <t>Cuộc họp A (24/8/2026)</t>
-  </si>
-  <si>
-    <t>Chủ trì xã Test</t>
-  </si>
-  <si>
-    <t>Đại biểu HĐND xã Test</t>
-  </si>
-  <si>
-    <t>Đại biểu HĐND xã Test 2</t>
-  </si>
-  <si>
-    <t>Đại biểu xã 3</t>
-  </si>
-  <si>
-    <t>Đại biểu xã 4</t>
-  </si>
-  <si>
-    <t>Đại biểu xã 5</t>
-  </si>
-  <si>
-    <t>Đại biểu xã 6</t>
-  </si>
-  <si>
-    <t>Đại biểu xã 7</t>
+    <t>Cuộc họp tỉnh giả định (21/09/2026)</t>
+  </si>
+  <si>
+    <t>Chủ trì tỉnh</t>
+  </si>
+  <si>
+    <t>Chủ trì tỉnh 2</t>
+  </si>
+  <si>
+    <t>Chủ trì tỉnh 3</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 1</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 2</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 3</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 4</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 5</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 6</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 7</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 8</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 9</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 10</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 11</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 12</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 13</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 14</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 15</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 16</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 17</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 18</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 19</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 20</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 21</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 22</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 23</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 24</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 25</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 26</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 27</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 28</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 29</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 30</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 31</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 32</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 33</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 34</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 35</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 36</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 37</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 38</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 39</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 40</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 41</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 42</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 43</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 44</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 45</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 46</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 47</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 48</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 49</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 50</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 51</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 52</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 53</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 54</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 55</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 56</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 57</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 58</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 59</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 60</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 61</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 62</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 63</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 64</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 65</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 66</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 67</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 68</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 69</t>
+  </si>
+  <si>
+    <t>Đại biểu tỉnh 70</t>
   </si>
 </sst>
 </file>
@@ -441,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521E990C-44C3-4D53-942C-AE6C6FB0D600}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -521,7 +716,527 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B31" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B32" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B36" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B38" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B40" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B41" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B43" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B44" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B45" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B50" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B52" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B53" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B55" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B56" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B62" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B63" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B64" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B66" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B68" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B69" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B71" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B72" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B73" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B74" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>